<commit_message>
Added 09-13-2026 Results Pt 1
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -673,8 +673,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H6" s="1" t="n"/>
-      <c r="I6" s="1" t="n"/>
+      <c r="H6" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>26</v>
+      </c>
       <c r="J6" s="1" t="n">
         <v>0</v>
       </c>
@@ -711,8 +715,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H7" s="1" t="n"/>
-      <c r="I7" s="1" t="n"/>
+      <c r="H7" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>14</v>
+      </c>
       <c r="J7" s="1" t="n">
         <v>0</v>
       </c>
@@ -749,8 +757,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H8" s="1" t="n"/>
-      <c r="I8" s="1" t="n"/>
+      <c r="H8" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J8" s="1" t="n">
         <v>0</v>
       </c>
@@ -787,8 +799,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H9" s="1" t="n"/>
-      <c r="I9" s="1" t="n"/>
+      <c r="H9" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J9" s="1" t="n">
         <v>0</v>
       </c>
@@ -825,8 +841,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H10" s="1" t="n"/>
-      <c r="I10" s="1" t="n"/>
+      <c r="H10" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>41</v>
+      </c>
       <c r="J10" s="1" t="n">
         <v>0</v>
       </c>
@@ -863,8 +883,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H11" s="1" t="n"/>
-      <c r="I11" s="1" t="n"/>
+      <c r="H11" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="I11" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J11" s="1" t="n">
         <v>0</v>
       </c>
@@ -901,8 +925,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H12" s="1" t="n"/>
-      <c r="I12" s="1" t="n"/>
+      <c r="H12" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I12" s="1" t="n">
+        <v>36</v>
+      </c>
       <c r="J12" s="1" t="n">
         <v>0</v>
       </c>
@@ -939,8 +967,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n"/>
-      <c r="I13" s="1" t="n"/>
+      <c r="H13" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="I13" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J13" s="1" t="n">
         <v>0</v>
       </c>
@@ -977,8 +1009,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H14" s="1" t="n"/>
-      <c r="I14" s="1" t="n"/>
+      <c r="H14" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="I14" s="1" t="n">
+        <v>59</v>
+      </c>
       <c r="J14" s="1" t="n">
         <v>0</v>
       </c>
@@ -1015,8 +1051,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H15" s="1" t="n"/>
-      <c r="I15" s="1" t="n"/>
+      <c r="H15" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="I15" s="1" t="n">
+        <v>37</v>
+      </c>
       <c r="J15" s="1" t="n">
         <v>0</v>
       </c>
@@ -1053,8 +1093,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H16" s="1" t="n"/>
-      <c r="I16" s="1" t="n"/>
+      <c r="H16" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="I16" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J16" s="1" t="n">
         <v>0</v>
       </c>
@@ -1091,8 +1135,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H17" s="1" t="n"/>
-      <c r="I17" s="1" t="n"/>
+      <c r="H17" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I17" s="1" t="n">
+        <v>33</v>
+      </c>
       <c r="J17" s="1" t="n">
         <v>0</v>
       </c>
@@ -1129,8 +1177,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H18" s="1" t="n"/>
-      <c r="I18" s="1" t="n"/>
+      <c r="H18" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="I18" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="J18" s="1" t="n">
         <v>0</v>
       </c>
@@ -1167,8 +1219,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H19" s="1" t="n"/>
-      <c r="I19" s="1" t="n"/>
+      <c r="H19" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>34</v>
+      </c>
       <c r="J19" s="1" t="n">
         <v>0</v>
       </c>
@@ -1281,10 +1337,14 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H22" s="1" t="n"/>
-      <c r="I22" s="1" t="n"/>
+      <c r="H22" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I22" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J22" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" ht="15.5" customHeight="1">
@@ -1319,10 +1379,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H23" s="1" t="n"/>
-      <c r="I23" s="1" t="n"/>
+      <c r="H23" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I23" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J23" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" ht="15.5" customHeight="1">
@@ -1433,8 +1497,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H26" s="1" t="n"/>
-      <c r="I26" s="1" t="n"/>
+      <c r="H26" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I26" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J26" s="1" t="n">
         <v>0</v>
       </c>
@@ -1471,8 +1539,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H27" s="1" t="n"/>
-      <c r="I27" s="1" t="n"/>
+      <c r="H27" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I27" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J27" s="1" t="n">
         <v>0</v>
       </c>
@@ -1509,8 +1581,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H28" s="1" t="n"/>
-      <c r="I28" s="1" t="n"/>
+      <c r="H28" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I28" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J28" s="1" t="n">
         <v>0</v>
       </c>
@@ -1547,8 +1623,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H29" s="1" t="n"/>
-      <c r="I29" s="1" t="n"/>
+      <c r="H29" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I29" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="J29" s="1" t="n">
         <v>0</v>
       </c>
@@ -1585,8 +1665,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H30" s="1" t="n"/>
-      <c r="I30" s="1" t="n"/>
+      <c r="H30" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I30" s="1" t="n">
+        <v>22</v>
+      </c>
       <c r="J30" s="1" t="n">
         <v>0</v>
       </c>
@@ -1623,8 +1707,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H31" s="1" t="n"/>
-      <c r="I31" s="1" t="n"/>
+      <c r="H31" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="I31" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J31" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added 09-13-2026 Results Pt 2
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -1421,8 +1421,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H24" s="1" t="n"/>
-      <c r="I24" s="1" t="n"/>
+      <c r="H24" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="I24" s="1" t="n">
+        <v>22</v>
+      </c>
       <c r="J24" s="1" t="n">
         <v>0</v>
       </c>
@@ -1459,8 +1463,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H25" s="1" t="n"/>
-      <c r="I25" s="1" t="n"/>
+      <c r="H25" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="I25" s="1" t="n">
+        <v>39</v>
+      </c>
       <c r="J25" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added 09-13-2026 Results Pt 3
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -1261,8 +1261,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H20" s="1" t="n"/>
-      <c r="I20" s="1" t="n"/>
+      <c r="H20" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="I20" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J20" s="1" t="n">
         <v>0</v>
       </c>
@@ -1299,8 +1303,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H21" s="1" t="n"/>
-      <c r="I21" s="1" t="n"/>
+      <c r="H21" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I21" s="1" t="n">
+        <v>28</v>
+      </c>
       <c r="J21" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added Week 2 Results and WNBA Update
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -1849,8 +1849,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H34" s="1" t="n"/>
-      <c r="I34" s="1" t="n"/>
+      <c r="H34" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="I34" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J34" s="1" t="n">
         <v>0</v>
       </c>
@@ -1887,8 +1891,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H35" s="1" t="n"/>
-      <c r="I35" s="1" t="n"/>
+      <c r="H35" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I35" s="1" t="n">
+        <v>41</v>
+      </c>
       <c r="J35" s="1" t="n">
         <v>0</v>
       </c>
@@ -1925,8 +1933,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H36" s="1" t="n"/>
-      <c r="I36" s="1" t="n"/>
+      <c r="H36" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I36" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J36" s="1" t="n">
         <v>0</v>
       </c>
@@ -1963,8 +1975,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H37" s="1" t="n"/>
-      <c r="I37" s="1" t="n"/>
+      <c r="H37" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I37" s="1" t="n">
+        <v>7</v>
+      </c>
       <c r="J37" s="1" t="n">
         <v>0</v>
       </c>
@@ -2001,8 +2017,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H38" s="1" t="n"/>
-      <c r="I38" s="1" t="n"/>
+      <c r="H38" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I38" s="1" t="n">
+        <v>34</v>
+      </c>
       <c r="J38" s="1" t="n">
         <v>0</v>
       </c>
@@ -2039,8 +2059,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H39" s="1" t="n"/>
-      <c r="I39" s="1" t="n"/>
+      <c r="H39" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="I39" s="1" t="n">
+        <v>3</v>
+      </c>
       <c r="J39" s="1" t="n">
         <v>0</v>
       </c>
@@ -2077,8 +2101,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H40" s="1" t="n"/>
-      <c r="I40" s="1" t="n"/>
+      <c r="H40" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I40" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J40" s="1" t="n">
         <v>0</v>
       </c>
@@ -2115,8 +2143,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H41" s="1" t="n"/>
-      <c r="I41" s="1" t="n"/>
+      <c r="H41" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I41" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J41" s="1" t="n">
         <v>0</v>
       </c>
@@ -2153,8 +2185,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H42" s="1" t="n"/>
-      <c r="I42" s="1" t="n"/>
+      <c r="H42" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I42" s="1" t="n">
+        <v>9</v>
+      </c>
       <c r="J42" s="1" t="n">
         <v>0</v>
       </c>
@@ -2191,8 +2227,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H43" s="1" t="n"/>
-      <c r="I43" s="1" t="n"/>
+      <c r="H43" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="I43" s="1" t="n">
+        <v>3</v>
+      </c>
       <c r="J43" s="1" t="n">
         <v>0</v>
       </c>
@@ -2229,8 +2269,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H44" s="1" t="n"/>
-      <c r="I44" s="1" t="n"/>
+      <c r="H44" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I44" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J44" s="1" t="n">
         <v>0</v>
       </c>
@@ -2267,8 +2311,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H45" s="1" t="n"/>
-      <c r="I45" s="1" t="n"/>
+      <c r="H45" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I45" s="1" t="n">
+        <v>6</v>
+      </c>
       <c r="J45" s="1" t="n">
         <v>0</v>
       </c>
@@ -2305,8 +2353,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H46" s="1" t="n"/>
-      <c r="I46" s="1" t="n"/>
+      <c r="H46" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I46" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J46" s="1" t="n">
         <v>0</v>
       </c>
@@ -2343,8 +2395,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H47" s="1" t="n"/>
-      <c r="I47" s="1" t="n"/>
+      <c r="H47" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I47" s="1" t="n">
+        <v>19</v>
+      </c>
       <c r="J47" s="1" t="n">
         <v>0</v>
       </c>
@@ -2381,8 +2437,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H48" s="1" t="n"/>
-      <c r="I48" s="1" t="n"/>
+      <c r="H48" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="I48" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J48" s="1" t="n">
         <v>0</v>
       </c>
@@ -2419,8 +2479,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H49" s="1" t="n"/>
-      <c r="I49" s="1" t="n"/>
+      <c r="H49" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I49" s="1" t="n">
+        <v>37</v>
+      </c>
       <c r="J49" s="1" t="n">
         <v>0</v>
       </c>
@@ -2457,8 +2521,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H50" s="1" t="n"/>
-      <c r="I50" s="1" t="n"/>
+      <c r="H50" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I50" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J50" s="1" t="n">
         <v>0</v>
       </c>
@@ -2495,8 +2563,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H51" s="1" t="n"/>
-      <c r="I51" s="1" t="n"/>
+      <c r="H51" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I51" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J51" s="1" t="n">
         <v>0</v>
       </c>
@@ -2533,10 +2605,14 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H52" s="1" t="n"/>
-      <c r="I52" s="1" t="n"/>
+      <c r="H52" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I52" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J52" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="15.5" customHeight="1">
@@ -2571,10 +2647,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H53" s="1" t="n"/>
-      <c r="I53" s="1" t="n"/>
+      <c r="H53" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I53" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J53" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" ht="15.5" customHeight="1">
@@ -2609,10 +2689,14 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H54" s="1" t="n"/>
-      <c r="I54" s="1" t="n"/>
+      <c r="H54" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="I54" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J54" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" ht="15.5" customHeight="1">
@@ -2647,10 +2731,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H55" s="1" t="n"/>
-      <c r="I55" s="1" t="n"/>
+      <c r="H55" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I55" s="1" t="n">
+        <v>33</v>
+      </c>
       <c r="J55" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" ht="15.5" customHeight="1">
@@ -2685,8 +2773,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H56" s="1" t="n"/>
-      <c r="I56" s="1" t="n"/>
+      <c r="H56" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I56" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J56" s="1" t="n">
         <v>0</v>
       </c>
@@ -2723,8 +2815,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H57" s="1" t="n"/>
-      <c r="I57" s="1" t="n"/>
+      <c r="H57" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I57" s="1" t="n">
+        <v>35</v>
+      </c>
       <c r="J57" s="1" t="n">
         <v>0</v>
       </c>
@@ -2761,8 +2857,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H58" s="1" t="n"/>
-      <c r="I58" s="1" t="n"/>
+      <c r="H58" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I58" s="1" t="n">
+        <v>3</v>
+      </c>
       <c r="J58" s="1" t="n">
         <v>0</v>
       </c>
@@ -2799,8 +2899,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H59" s="1" t="n"/>
-      <c r="I59" s="1" t="n"/>
+      <c r="H59" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I59" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J59" s="1" t="n">
         <v>0</v>
       </c>
@@ -2837,8 +2941,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H60" s="1" t="n"/>
-      <c r="I60" s="1" t="n"/>
+      <c r="H60" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="I60" s="1" t="n">
+        <v>26</v>
+      </c>
       <c r="J60" s="1" t="n">
         <v>0</v>
       </c>
@@ -2875,8 +2983,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H61" s="1" t="n"/>
-      <c r="I61" s="1" t="n"/>
+      <c r="H61" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="I61" s="1" t="n">
+        <v>14</v>
+      </c>
       <c r="J61" s="1" t="n">
         <v>0</v>
       </c>
@@ -2913,8 +3025,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H62" s="1" t="n"/>
-      <c r="I62" s="1" t="n"/>
+      <c r="H62" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I62" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J62" s="1" t="n">
         <v>0</v>
       </c>
@@ -2951,8 +3067,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H63" s="1" t="n"/>
-      <c r="I63" s="1" t="n"/>
+      <c r="H63" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I63" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J63" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added 9-24-2026 NFL Results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -3109,8 +3109,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H64" s="1" t="n"/>
-      <c r="I64" s="1" t="n"/>
+      <c r="H64" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="I64" s="1" t="n">
+        <v>6</v>
+      </c>
       <c r="J64" s="1" t="n">
         <v>0</v>
       </c>
@@ -3147,8 +3151,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H65" s="1" t="n"/>
-      <c r="I65" s="1" t="n"/>
+      <c r="H65" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I65" s="1" t="n">
+        <v>28</v>
+      </c>
       <c r="J65" s="1" t="n">
         <v>0</v>
       </c>
@@ -3185,8 +3193,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H66" s="1" t="n"/>
-      <c r="I66" s="1" t="n"/>
+      <c r="H66" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="I66" s="1" t="n">
+        <v>35</v>
+      </c>
       <c r="J66" s="1" t="n">
         <v>0</v>
       </c>
@@ -3223,8 +3235,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H67" s="1" t="n"/>
-      <c r="I67" s="1" t="n"/>
+      <c r="H67" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I67" s="1" t="n">
+        <v>14</v>
+      </c>
       <c r="J67" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Updated WNBA and NFL Results for 9-27-2026
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -3277,8 +3277,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H68" s="1" t="n"/>
-      <c r="I68" s="1" t="n"/>
+      <c r="H68" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="I68" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J68" s="1" t="n">
         <v>0</v>
       </c>
@@ -3315,8 +3319,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H69" s="1" t="n"/>
-      <c r="I69" s="1" t="n"/>
+      <c r="H69" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I69" s="1" t="n">
+        <v>36</v>
+      </c>
       <c r="J69" s="1" t="n">
         <v>0</v>
       </c>
@@ -3353,8 +3361,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H70" s="1" t="n"/>
-      <c r="I70" s="1" t="n"/>
+      <c r="H70" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="I70" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J70" s="1" t="n">
         <v>0</v>
       </c>
@@ -3391,8 +3403,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H71" s="1" t="n"/>
-      <c r="I71" s="1" t="n"/>
+      <c r="H71" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I71" s="1" t="n">
+        <v>34</v>
+      </c>
       <c r="J71" s="1" t="n">
         <v>0</v>
       </c>
@@ -3429,8 +3445,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H72" s="1" t="n"/>
-      <c r="I72" s="1" t="n"/>
+      <c r="H72" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I72" s="1" t="n">
+        <v>16</v>
+      </c>
       <c r="J72" s="1" t="n">
         <v>0</v>
       </c>
@@ -3467,8 +3487,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H73" s="1" t="n"/>
-      <c r="I73" s="1" t="n"/>
+      <c r="H73" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="I73" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J73" s="1" t="n">
         <v>0</v>
       </c>
@@ -3505,8 +3529,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H74" s="1" t="n"/>
-      <c r="I74" s="1" t="n"/>
+      <c r="H74" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="I74" s="1" t="n">
+        <v>18</v>
+      </c>
       <c r="J74" s="1" t="n">
         <v>0</v>
       </c>
@@ -3543,8 +3571,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H75" s="1" t="n"/>
-      <c r="I75" s="1" t="n"/>
+      <c r="H75" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="I75" s="1" t="n">
+        <v>21</v>
+      </c>
       <c r="J75" s="1" t="n">
         <v>0</v>
       </c>
@@ -3581,8 +3613,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H76" s="1" t="n"/>
-      <c r="I76" s="1" t="n"/>
+      <c r="H76" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I76" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J76" s="1" t="n">
         <v>0</v>
       </c>
@@ -3619,8 +3655,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H77" s="1" t="n"/>
-      <c r="I77" s="1" t="n"/>
+      <c r="H77" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I77" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J77" s="1" t="n">
         <v>0</v>
       </c>
@@ -3657,8 +3697,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H78" s="1" t="n"/>
-      <c r="I78" s="1" t="n"/>
+      <c r="H78" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I78" s="1" t="n">
+        <v>26</v>
+      </c>
       <c r="J78" s="1" t="n">
         <v>0</v>
       </c>
@@ -3695,8 +3739,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H79" s="1" t="n"/>
-      <c r="I79" s="1" t="n"/>
+      <c r="H79" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="I79" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J79" s="1" t="n">
         <v>0</v>
       </c>
@@ -3733,8 +3781,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H80" s="1" t="n"/>
-      <c r="I80" s="1" t="n"/>
+      <c r="H80" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I80" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J80" s="1" t="n">
         <v>0</v>
       </c>
@@ -3771,8 +3823,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H81" s="1" t="n"/>
-      <c r="I81" s="1" t="n"/>
+      <c r="H81" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I81" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J81" s="1" t="n">
         <v>0</v>
       </c>
@@ -3809,8 +3865,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H82" s="1" t="n"/>
-      <c r="I82" s="1" t="n"/>
+      <c r="H82" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I82" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J82" s="1" t="n">
         <v>0</v>
       </c>
@@ -3847,8 +3907,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H83" s="1" t="n"/>
-      <c r="I83" s="1" t="n"/>
+      <c r="H83" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I83" s="1" t="n">
+        <v>19</v>
+      </c>
       <c r="J83" s="1" t="n">
         <v>0</v>
       </c>
@@ -3885,8 +3949,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H84" s="1" t="n"/>
-      <c r="I84" s="1" t="n"/>
+      <c r="H84" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I84" s="1" t="n">
+        <v>6</v>
+      </c>
       <c r="J84" s="1" t="n">
         <v>0</v>
       </c>
@@ -3923,8 +3991,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H85" s="1" t="n"/>
-      <c r="I85" s="1" t="n"/>
+      <c r="H85" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I85" s="1" t="n">
+        <v>35</v>
+      </c>
       <c r="J85" s="1" t="n">
         <v>0</v>
       </c>
@@ -3961,8 +4033,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H86" s="1" t="n"/>
-      <c r="I86" s="1" t="n"/>
+      <c r="H86" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I86" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J86" s="1" t="n">
         <v>0</v>
       </c>
@@ -3999,8 +4075,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H87" s="1" t="n"/>
-      <c r="I87" s="1" t="n"/>
+      <c r="H87" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I87" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="J87" s="1" t="n">
         <v>0</v>
       </c>
@@ -4037,8 +4117,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H88" s="1" t="n"/>
-      <c r="I88" s="1" t="n"/>
+      <c r="H88" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="I88" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J88" s="1" t="n">
         <v>0</v>
       </c>
@@ -4075,8 +4159,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H89" s="1" t="n"/>
-      <c r="I89" s="1" t="n"/>
+      <c r="H89" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I89" s="1" t="n">
+        <v>16</v>
+      </c>
       <c r="J89" s="1" t="n">
         <v>0</v>
       </c>
@@ -4113,8 +4201,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H90" s="1" t="n"/>
-      <c r="I90" s="1" t="n"/>
+      <c r="H90" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I90" s="1" t="n">
+        <v>35</v>
+      </c>
       <c r="J90" s="1" t="n">
         <v>0</v>
       </c>
@@ -4151,8 +4243,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H91" s="1" t="n"/>
-      <c r="I91" s="1" t="n"/>
+      <c r="H91" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I91" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J91" s="1" t="n">
         <v>0</v>
       </c>
@@ -4189,8 +4285,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H92" s="1" t="n"/>
-      <c r="I92" s="1" t="n"/>
+      <c r="H92" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="I92" s="1" t="n">
+        <v>7</v>
+      </c>
       <c r="J92" s="1" t="n">
         <v>0</v>
       </c>
@@ -4227,8 +4327,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H93" s="1" t="n"/>
-      <c r="I93" s="1" t="n"/>
+      <c r="H93" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I93" s="1" t="n">
+        <v>12</v>
+      </c>
       <c r="J93" s="1" t="n">
         <v>0</v>
       </c>
@@ -4265,8 +4369,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H94" s="1" t="n"/>
-      <c r="I94" s="1" t="n"/>
+      <c r="H94" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="I94" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J94" s="1" t="n">
         <v>0</v>
       </c>
@@ -4303,8 +4411,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H95" s="1" t="n"/>
-      <c r="I95" s="1" t="n"/>
+      <c r="H95" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I95" s="1" t="n">
+        <v>33</v>
+      </c>
       <c r="J95" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Updated NFL Results for 9-28-2026
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -4453,8 +4453,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H96" s="1" t="n"/>
-      <c r="I96" s="1" t="n"/>
+      <c r="H96" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I96" s="1" t="n">
+        <v>7</v>
+      </c>
       <c r="J96" s="1" t="n">
         <v>0</v>
       </c>
@@ -4491,8 +4495,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H97" s="1" t="n"/>
-      <c r="I97" s="1" t="n"/>
+      <c r="H97" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I97" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J97" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for 10-1-2026
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -4537,8 +4537,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H98" s="1" t="n"/>
-      <c r="I98" s="1" t="n"/>
+      <c r="H98" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I98" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J98" s="1" t="n">
         <v>0</v>
       </c>
@@ -4575,8 +4579,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H99" s="1" t="n"/>
-      <c r="I99" s="1" t="n"/>
+      <c r="H99" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I99" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J99" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for 10-4-2026
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -4621,8 +4621,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H100" s="1" t="n"/>
-      <c r="I100" s="1" t="n"/>
+      <c r="H100" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="I100" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J100" s="1" t="n">
         <v>0</v>
       </c>
@@ -4659,8 +4663,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H101" s="1" t="n"/>
-      <c r="I101" s="1" t="n"/>
+      <c r="H101" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I101" s="1" t="n">
+        <v>36</v>
+      </c>
       <c r="J101" s="1" t="n">
         <v>0</v>
       </c>
@@ -4697,8 +4705,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H102" s="1" t="n"/>
-      <c r="I102" s="1" t="n"/>
+      <c r="H102" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I102" s="1" t="n">
+        <v>18</v>
+      </c>
       <c r="J102" s="1" t="n">
         <v>0</v>
       </c>
@@ -4735,8 +4747,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H103" s="1" t="n"/>
-      <c r="I103" s="1" t="n"/>
+      <c r="H103" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="I103" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J103" s="1" t="n">
         <v>0</v>
       </c>
@@ -4773,8 +4789,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H104" s="1" t="n"/>
-      <c r="I104" s="1" t="n"/>
+      <c r="H104" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="I104" s="1" t="n">
+        <v>29</v>
+      </c>
       <c r="J104" s="1" t="n">
         <v>0</v>
       </c>
@@ -4811,8 +4831,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H105" s="1" t="n"/>
-      <c r="I105" s="1" t="n"/>
+      <c r="H105" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="I105" s="1" t="n">
+        <v>26</v>
+      </c>
       <c r="J105" s="1" t="n">
         <v>0</v>
       </c>
@@ -4849,8 +4873,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H106" s="1" t="n"/>
-      <c r="I106" s="1" t="n"/>
+      <c r="H106" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="I106" s="1" t="n">
+        <v>26</v>
+      </c>
       <c r="J106" s="1" t="n">
         <v>0</v>
       </c>
@@ -4887,8 +4915,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H107" s="1" t="n"/>
-      <c r="I107" s="1" t="n"/>
+      <c r="H107" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="I107" s="1" t="n">
+        <v>32</v>
+      </c>
       <c r="J107" s="1" t="n">
         <v>0</v>
       </c>
@@ -4925,8 +4957,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H108" s="1" t="n"/>
-      <c r="I108" s="1" t="n"/>
+      <c r="H108" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I108" s="1" t="n">
+        <v>12</v>
+      </c>
       <c r="J108" s="1" t="n">
         <v>0</v>
       </c>
@@ -4963,8 +4999,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H109" s="1" t="n"/>
-      <c r="I109" s="1" t="n"/>
+      <c r="H109" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="I109" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J109" s="1" t="n">
         <v>0</v>
       </c>
@@ -5001,8 +5041,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H110" s="1" t="n"/>
-      <c r="I110" s="1" t="n"/>
+      <c r="H110" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I110" s="1" t="n">
+        <v>22</v>
+      </c>
       <c r="J110" s="1" t="n">
         <v>0</v>
       </c>
@@ -5039,8 +5083,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H111" s="1" t="n"/>
-      <c r="I111" s="1" t="n"/>
+      <c r="H111" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="I111" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J111" s="1" t="n">
         <v>0</v>
       </c>
@@ -5077,8 +5125,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H112" s="1" t="n"/>
-      <c r="I112" s="1" t="n"/>
+      <c r="H112" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I112" s="1" t="n">
+        <v>34</v>
+      </c>
       <c r="J112" s="1" t="n">
         <v>0</v>
       </c>
@@ -5115,8 +5167,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H113" s="1" t="n"/>
-      <c r="I113" s="1" t="n"/>
+      <c r="H113" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="I113" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J113" s="1" t="n">
         <v>0</v>
       </c>
@@ -5153,8 +5209,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H114" s="1" t="n"/>
-      <c r="I114" s="1" t="n"/>
+      <c r="H114" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I114" s="1" t="n">
+        <v>14</v>
+      </c>
       <c r="J114" s="1" t="n">
         <v>0</v>
       </c>
@@ -5191,8 +5251,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H115" s="1" t="n"/>
-      <c r="I115" s="1" t="n"/>
+      <c r="H115" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="I115" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J115" s="1" t="n">
         <v>0</v>
       </c>
@@ -5229,8 +5293,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H116" s="1" t="n"/>
-      <c r="I116" s="1" t="n"/>
+      <c r="H116" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="I116" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J116" s="1" t="n">
         <v>0</v>
       </c>
@@ -5267,8 +5335,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H117" s="1" t="n"/>
-      <c r="I117" s="1" t="n"/>
+      <c r="H117" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I117" s="1" t="n">
+        <v>14</v>
+      </c>
       <c r="J117" s="1" t="n">
         <v>0</v>
       </c>
@@ -5305,8 +5377,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H118" s="1" t="n"/>
-      <c r="I118" s="1" t="n"/>
+      <c r="H118" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I118" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J118" s="1" t="n">
         <v>0</v>
       </c>
@@ -5343,8 +5419,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H119" s="1" t="n"/>
-      <c r="I119" s="1" t="n"/>
+      <c r="H119" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I119" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J119" s="1" t="n">
         <v>0</v>
       </c>
@@ -5381,8 +5461,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H120" s="1" t="n"/>
-      <c r="I120" s="1" t="n"/>
+      <c r="H120" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I120" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J120" s="1" t="n">
         <v>0</v>
       </c>
@@ -5419,8 +5503,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H121" s="1" t="n"/>
-      <c r="I121" s="1" t="n"/>
+      <c r="H121" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I121" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J121" s="1" t="n">
         <v>0</v>
       </c>
@@ -5457,8 +5545,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H122" s="1" t="n"/>
-      <c r="I122" s="1" t="n"/>
+      <c r="H122" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="I122" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="J122" s="1" t="n">
         <v>0</v>
       </c>
@@ -5495,8 +5587,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H123" s="1" t="n"/>
-      <c r="I123" s="1" t="n"/>
+      <c r="H123" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I123" s="1" t="n">
+        <v>15</v>
+      </c>
       <c r="J123" s="1" t="n">
         <v>0</v>
       </c>
@@ -5533,8 +5629,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H124" s="1" t="n"/>
-      <c r="I124" s="1" t="n"/>
+      <c r="H124" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I124" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J124" s="1" t="n">
         <v>0</v>
       </c>
@@ -5571,8 +5671,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H125" s="1" t="n"/>
-      <c r="I125" s="1" t="n"/>
+      <c r="H125" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I125" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J125" s="1" t="n">
         <v>0</v>
       </c>
@@ -5609,8 +5713,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H126" s="1" t="n"/>
-      <c r="I126" s="1" t="n"/>
+      <c r="H126" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I126" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J126" s="1" t="n">
         <v>0</v>
       </c>
@@ -5647,8 +5755,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H127" s="1" t="n"/>
-      <c r="I127" s="1" t="n"/>
+      <c r="H127" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I127" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J127" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for 10-5-2026
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -5797,8 +5797,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H128" s="1" t="n"/>
-      <c r="I128" s="1" t="n"/>
+      <c r="H128" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I128" s="1" t="n">
+        <v>45</v>
+      </c>
       <c r="J128" s="1" t="n">
         <v>0</v>
       </c>
@@ -5835,8 +5839,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H129" s="1" t="n"/>
-      <c r="I129" s="1" t="n"/>
+      <c r="H129" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="I129" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J129" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added 10-8-2026 NFL Results
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -5881,8 +5881,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H130" s="1" t="n"/>
-      <c r="I130" s="1" t="n"/>
+      <c r="H130" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="I130" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J130" s="1" t="n">
         <v>0</v>
       </c>
@@ -5919,8 +5923,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H131" s="1" t="n"/>
-      <c r="I131" s="1" t="n"/>
+      <c r="H131" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I131" s="1" t="n">
+        <v>16</v>
+      </c>
       <c r="J131" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 10, 2026 - Part 1
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NFL_2026_Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="NFL_2026_Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Added NFL Results for Oct 11, 2026 - Part 1
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -6117,8 +6117,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H136" s="1" t="n"/>
-      <c r="I136" s="1" t="n"/>
+      <c r="H136" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I136" s="1" t="n">
+        <v>7</v>
+      </c>
       <c r="J136" s="1" t="n">
         <v>0</v>
       </c>
@@ -6155,8 +6159,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H137" s="1" t="n"/>
-      <c r="I137" s="1" t="n"/>
+      <c r="H137" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="I137" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J137" s="1" t="n">
         <v>0</v>
       </c>
@@ -6193,8 +6201,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H138" s="1" t="n"/>
-      <c r="I138" s="1" t="n"/>
+      <c r="H138" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I138" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J138" s="1" t="n">
         <v>0</v>
       </c>
@@ -6231,8 +6243,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H139" s="1" t="n"/>
-      <c r="I139" s="1" t="n"/>
+      <c r="H139" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I139" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J139" s="1" t="n">
         <v>0</v>
       </c>
@@ -6269,8 +6285,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H140" s="1" t="n"/>
-      <c r="I140" s="1" t="n"/>
+      <c r="H140" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I140" s="1" t="n">
+        <v>12</v>
+      </c>
       <c r="J140" s="1" t="n">
         <v>0</v>
       </c>
@@ -6307,8 +6327,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H141" s="1" t="n"/>
-      <c r="I141" s="1" t="n"/>
+      <c r="H141" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="I141" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J141" s="1" t="n">
         <v>0</v>
       </c>
@@ -6421,8 +6445,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H144" s="1" t="n"/>
-      <c r="I144" s="1" t="n"/>
+      <c r="H144" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I144" s="1" t="n">
+        <v>26</v>
+      </c>
       <c r="J144" s="1" t="n">
         <v>0</v>
       </c>
@@ -6459,8 +6487,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H145" s="1" t="n"/>
-      <c r="I145" s="1" t="n"/>
+      <c r="H145" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="I145" s="1" t="n">
+        <v>3</v>
+      </c>
       <c r="J145" s="1" t="n">
         <v>0</v>
       </c>
@@ -6497,8 +6529,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H146" s="1" t="n"/>
-      <c r="I146" s="1" t="n"/>
+      <c r="H146" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="I146" s="1" t="n">
+        <v>22</v>
+      </c>
       <c r="J146" s="1" t="n">
         <v>0</v>
       </c>
@@ -6535,8 +6571,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H147" s="1" t="n"/>
-      <c r="I147" s="1" t="n"/>
+      <c r="H147" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="I147" s="1" t="n">
+        <v>34</v>
+      </c>
       <c r="J147" s="1" t="n">
         <v>0</v>
       </c>
@@ -6573,8 +6613,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H148" s="1" t="n"/>
-      <c r="I148" s="1" t="n"/>
+      <c r="H148" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I148" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J148" s="1" t="n">
         <v>0</v>
       </c>
@@ -6611,8 +6655,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H149" s="1" t="n"/>
-      <c r="I149" s="1" t="n"/>
+      <c r="H149" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I149" s="1" t="n">
+        <v>19</v>
+      </c>
       <c r="J149" s="1" t="n">
         <v>0</v>
       </c>
@@ -6649,8 +6697,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H150" s="1" t="n"/>
-      <c r="I150" s="1" t="n"/>
+      <c r="H150" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I150" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J150" s="1" t="n">
         <v>0</v>
       </c>
@@ -6687,8 +6739,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H151" s="1" t="n"/>
-      <c r="I151" s="1" t="n"/>
+      <c r="H151" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I151" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J151" s="1" t="n">
         <v>0</v>
       </c>
@@ -6725,8 +6781,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H152" s="1" t="n"/>
-      <c r="I152" s="1" t="n"/>
+      <c r="H152" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="I152" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J152" s="1" t="n">
         <v>0</v>
       </c>
@@ -6763,8 +6823,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H153" s="1" t="n"/>
-      <c r="I153" s="1" t="n"/>
+      <c r="H153" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I153" s="1" t="n">
+        <v>45</v>
+      </c>
       <c r="J153" s="1" t="n">
         <v>0</v>
       </c>
@@ -6801,10 +6865,14 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H154" s="1" t="n"/>
-      <c r="I154" s="1" t="n"/>
+      <c r="H154" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I154" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J154" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155" ht="15.5" customHeight="1">
@@ -6839,10 +6907,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H155" s="1" t="n"/>
-      <c r="I155" s="1" t="n"/>
+      <c r="H155" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I155" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J155" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156" ht="15.5" customHeight="1">

</xml_diff>

<commit_message>
Added NFL Results for Oct 11, 2026 - Part 3
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -5965,8 +5965,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H132" s="1" t="n"/>
-      <c r="I132" s="1" t="n"/>
+      <c r="H132" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="I132" s="1" t="n">
+        <v>45</v>
+      </c>
       <c r="J132" s="1" t="n">
         <v>0</v>
       </c>
@@ -6003,8 +6007,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H133" s="1" t="n"/>
-      <c r="I133" s="1" t="n"/>
+      <c r="H133" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="I133" s="1" t="n">
+        <v>21</v>
+      </c>
       <c r="J133" s="1" t="n">
         <v>0</v>
       </c>
@@ -6369,8 +6377,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H142" s="1" t="n"/>
-      <c r="I142" s="1" t="n"/>
+      <c r="H142" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I142" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J142" s="1" t="n">
         <v>0</v>
       </c>
@@ -6407,8 +6419,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H143" s="1" t="n"/>
-      <c r="I143" s="1" t="n"/>
+      <c r="H143" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I143" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J143" s="1" t="n">
         <v>0</v>
       </c>
@@ -6949,8 +6965,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H156" s="1" t="n"/>
-      <c r="I156" s="1" t="n"/>
+      <c r="H156" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="I156" s="1" t="n">
+        <v>32</v>
+      </c>
       <c r="J156" s="1" t="n">
         <v>0</v>
       </c>
@@ -6987,8 +7007,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H157" s="1" t="n"/>
-      <c r="I157" s="1" t="n"/>
+      <c r="H157" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="I157" s="1" t="n">
+        <v>29</v>
+      </c>
       <c r="J157" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 11, 2026 - Part 4
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -6049,10 +6049,14 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H134" s="1" t="n"/>
-      <c r="I134" s="1" t="n"/>
+      <c r="H134" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I134" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J134" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135" ht="15.5" customHeight="1">
@@ -6087,10 +6091,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H135" s="1" t="n"/>
-      <c r="I135" s="1" t="n"/>
+      <c r="H135" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I135" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J135" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136" ht="15.5" customHeight="1">

</xml_diff>

<commit_message>
Added NFL Results for Oct 12, 2026 - Part 3
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -7057,10 +7057,14 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H158" s="1" t="n"/>
-      <c r="I158" s="1" t="n"/>
+      <c r="H158" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="I158" s="1" t="n">
+        <v>37</v>
+      </c>
       <c r="J158" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159" ht="15.5" customHeight="1">
@@ -7095,10 +7099,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H159" s="1" t="n"/>
-      <c r="I159" s="1" t="n"/>
+      <c r="H159" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="I159" s="1" t="n">
+        <v>34</v>
+      </c>
       <c r="J159" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160" ht="15.5" customHeight="1">

</xml_diff>

<commit_message>
Added NFL Results for Oct 15, 2026 - Part 1
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -7141,10 +7141,14 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H160" s="1" t="n"/>
-      <c r="I160" s="1" t="n"/>
+      <c r="H160" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I160" s="1" t="n">
+        <v>14</v>
+      </c>
       <c r="J160" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161" ht="15.5" customHeight="1">
@@ -7179,10 +7183,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H161" s="1" t="n"/>
-      <c r="I161" s="1" t="n"/>
+      <c r="H161" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="I161" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J161" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162" ht="15.5" customHeight="1">

</xml_diff>

<commit_message>
Added NFL Results for Oct 18, 2026 - Part 1
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -7681,8 +7681,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H174" s="1" t="n"/>
-      <c r="I174" s="1" t="n"/>
+      <c r="H174" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="I174" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J174" s="1" t="n">
         <v>0</v>
       </c>
@@ -7719,8 +7723,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H175" s="1" t="n"/>
-      <c r="I175" s="1" t="n"/>
+      <c r="H175" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I175" s="1" t="n">
+        <v>34</v>
+      </c>
       <c r="J175" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 18, 2026 - Part 2
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -7301,8 +7301,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H164" s="1" t="n"/>
-      <c r="I164" s="1" t="n"/>
+      <c r="H164" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I164" s="1" t="n">
+        <v>31</v>
+      </c>
       <c r="J164" s="1" t="n">
         <v>0</v>
       </c>
@@ -7339,8 +7343,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H165" s="1" t="n"/>
-      <c r="I165" s="1" t="n"/>
+      <c r="H165" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="I165" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J165" s="1" t="n">
         <v>0</v>
       </c>
@@ -7377,8 +7385,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H166" s="1" t="n"/>
-      <c r="I166" s="1" t="n"/>
+      <c r="H166" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I166" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="J166" s="1" t="n">
         <v>0</v>
       </c>
@@ -7415,8 +7427,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H167" s="1" t="n"/>
-      <c r="I167" s="1" t="n"/>
+      <c r="H167" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I167" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J167" s="1" t="n">
         <v>0</v>
       </c>
@@ -7765,8 +7781,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H176" s="1" t="n"/>
-      <c r="I176" s="1" t="n"/>
+      <c r="H176" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I176" s="1" t="n">
+        <v>26</v>
+      </c>
       <c r="J176" s="1" t="n">
         <v>0</v>
       </c>
@@ -7803,8 +7823,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H177" s="1" t="n"/>
-      <c r="I177" s="1" t="n"/>
+      <c r="H177" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="I177" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J177" s="1" t="n">
         <v>0</v>
       </c>
@@ -7917,8 +7941,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H180" s="1" t="n"/>
-      <c r="I180" s="1" t="n"/>
+      <c r="H180" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="I180" s="1" t="n">
+        <v>19</v>
+      </c>
       <c r="J180" s="1" t="n">
         <v>0</v>
       </c>
@@ -7955,8 +7983,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H181" s="1" t="n"/>
-      <c r="I181" s="1" t="n"/>
+      <c r="H181" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I181" s="1" t="n">
+        <v>26</v>
+      </c>
       <c r="J181" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 18, 2026 - Part 3
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -7545,8 +7545,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H170" s="1" t="n"/>
-      <c r="I170" s="1" t="n"/>
+      <c r="H170" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="I170" s="1" t="n">
+        <v>25</v>
+      </c>
       <c r="J170" s="1" t="n">
         <v>0</v>
       </c>
@@ -7583,8 +7587,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H171" s="1" t="n"/>
-      <c r="I171" s="1" t="n"/>
+      <c r="H171" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="I171" s="1" t="n">
+        <v>14</v>
+      </c>
       <c r="J171" s="1" t="n">
         <v>0</v>
       </c>
@@ -8025,8 +8033,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H182" s="1" t="n"/>
-      <c r="I182" s="1" t="n"/>
+      <c r="H182" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I182" s="1" t="n">
+        <v>34</v>
+      </c>
       <c r="J182" s="1" t="n">
         <v>0</v>
       </c>
@@ -8063,8 +8075,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H183" s="1" t="n"/>
-      <c r="I183" s="1" t="n"/>
+      <c r="H183" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="I183" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J183" s="1" t="n">
         <v>0</v>
       </c>
@@ -8101,10 +8117,14 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H184" s="1" t="n"/>
-      <c r="I184" s="1" t="n"/>
+      <c r="H184" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I184" s="1" t="n">
+        <v>26</v>
+      </c>
       <c r="J184" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185" ht="15.5" customHeight="1">
@@ -8139,10 +8159,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H185" s="1" t="n"/>
-      <c r="I185" s="1" t="n"/>
+      <c r="H185" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="I185" s="1" t="n">
+        <v>19</v>
+      </c>
       <c r="J185" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="186" ht="15.5" customHeight="1">

</xml_diff>

<commit_message>
Added NFL Results for Oct 18, 2026 - Part 5
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -7225,8 +7225,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H162" s="1" t="n"/>
-      <c r="I162" s="1" t="n"/>
+      <c r="H162" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="I162" s="1" t="n">
+        <v>18</v>
+      </c>
       <c r="J162" s="1" t="n">
         <v>0</v>
       </c>
@@ -7263,8 +7267,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H163" s="1" t="n"/>
-      <c r="I163" s="1" t="n"/>
+      <c r="H163" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="I163" s="1" t="n">
+        <v>16</v>
+      </c>
       <c r="J163" s="1" t="n">
         <v>0</v>
       </c>
@@ -7469,8 +7477,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H168" s="1" t="n"/>
-      <c r="I168" s="1" t="n"/>
+      <c r="H168" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I168" s="1" t="n">
+        <v>33</v>
+      </c>
       <c r="J168" s="1" t="n">
         <v>0</v>
       </c>
@@ -7507,8 +7519,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H169" s="1" t="n"/>
-      <c r="I169" s="1" t="n"/>
+      <c r="H169" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="I169" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J169" s="1" t="n">
         <v>0</v>
       </c>
@@ -7873,8 +7889,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H178" s="1" t="n"/>
-      <c r="I178" s="1" t="n"/>
+      <c r="H178" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="I178" s="1" t="n">
+        <v>6</v>
+      </c>
       <c r="J178" s="1" t="n">
         <v>0</v>
       </c>
@@ -7911,8 +7931,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H179" s="1" t="n"/>
-      <c r="I179" s="1" t="n"/>
+      <c r="H179" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I179" s="1" t="n">
+        <v>22</v>
+      </c>
       <c r="J179" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 18, 2026 - Part 6
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -7645,8 +7645,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H172" s="1" t="n"/>
-      <c r="I172" s="1" t="n"/>
+      <c r="H172" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I172" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J172" s="1" t="n">
         <v>0</v>
       </c>
@@ -7683,8 +7687,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H173" s="1" t="n"/>
-      <c r="I173" s="1" t="n"/>
+      <c r="H173" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I173" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J173" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 19, 2026 - Part 3
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8233,8 +8233,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H186" s="1" t="n"/>
-      <c r="I186" s="1" t="n"/>
+      <c r="H186" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="I186" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J186" s="1" t="n">
         <v>0</v>
       </c>
@@ -8271,8 +8275,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H187" s="1" t="n"/>
-      <c r="I187" s="1" t="n"/>
+      <c r="H187" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I187" s="1" t="n">
+        <v>23</v>
+      </c>
       <c r="J187" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 22, 2026 - Part 1
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8317,8 +8317,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H188" s="1" t="n"/>
-      <c r="I188" s="1" t="n"/>
+      <c r="H188" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I188" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J188" s="1" t="n">
         <v>0</v>
       </c>
@@ -8355,8 +8359,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H189" s="1" t="n"/>
-      <c r="I189" s="1" t="n"/>
+      <c r="H189" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I189" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J189" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 25, 2026 - Part 1
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -9161,8 +9161,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H210" s="1" t="n"/>
-      <c r="I210" s="1" t="n"/>
+      <c r="H210" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I210" s="1" t="n">
+        <v>16</v>
+      </c>
       <c r="J210" s="1" t="n">
         <v>0</v>
       </c>
@@ -9199,8 +9203,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H211" s="1" t="n"/>
-      <c r="I211" s="1" t="n"/>
+      <c r="H211" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="I211" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="J211" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 25, 2026 - Part 2
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8477,8 +8477,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H192" s="1" t="n"/>
-      <c r="I192" s="1" t="n"/>
+      <c r="H192" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="I192" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J192" s="1" t="n">
         <v>0</v>
       </c>
@@ -8515,8 +8519,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H193" s="1" t="n"/>
-      <c r="I193" s="1" t="n"/>
+      <c r="H193" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I193" s="1" t="n">
+        <v>29</v>
+      </c>
       <c r="J193" s="1" t="n">
         <v>0</v>
       </c>
@@ -8553,8 +8561,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H194" s="1" t="n"/>
-      <c r="I194" s="1" t="n"/>
+      <c r="H194" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I194" s="1" t="n">
+        <v>35</v>
+      </c>
       <c r="J194" s="1" t="n">
         <v>0</v>
       </c>
@@ -8591,8 +8603,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H195" s="1" t="n"/>
-      <c r="I195" s="1" t="n"/>
+      <c r="H195" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I195" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J195" s="1" t="n">
         <v>0</v>
       </c>
@@ -8629,8 +8645,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H196" s="1" t="n"/>
-      <c r="I196" s="1" t="n"/>
+      <c r="H196" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="I196" s="1" t="n">
+        <v>43</v>
+      </c>
       <c r="J196" s="1" t="n">
         <v>0</v>
       </c>
@@ -8667,8 +8687,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H197" s="1" t="n"/>
-      <c r="I197" s="1" t="n"/>
+      <c r="H197" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="I197" s="1" t="n">
+        <v>13</v>
+      </c>
       <c r="J197" s="1" t="n">
         <v>0</v>
       </c>
@@ -8705,8 +8729,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H198" s="1" t="n"/>
-      <c r="I198" s="1" t="n"/>
+      <c r="H198" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="I198" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J198" s="1" t="n">
         <v>0</v>
       </c>
@@ -8743,8 +8771,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H199" s="1" t="n"/>
-      <c r="I199" s="1" t="n"/>
+      <c r="H199" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I199" s="1" t="n">
+        <v>24</v>
+      </c>
       <c r="J199" s="1" t="n">
         <v>0</v>
       </c>
@@ -8857,10 +8889,14 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H202" s="1" t="n"/>
-      <c r="I202" s="1" t="n"/>
+      <c r="H202" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="I202" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J202" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="203" ht="15.5" customHeight="1">
@@ -8895,10 +8931,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H203" s="1" t="n"/>
-      <c r="I203" s="1" t="n"/>
+      <c r="H203" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I203" s="1" t="n">
+        <v>21</v>
+      </c>
       <c r="J203" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="204" ht="15.5" customHeight="1">
@@ -8933,8 +8973,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H204" s="1" t="n"/>
-      <c r="I204" s="1" t="n"/>
+      <c r="H204" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="I204" s="1" t="n">
+        <v>10</v>
+      </c>
       <c r="J204" s="1" t="n">
         <v>0</v>
       </c>
@@ -8971,8 +9015,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H205" s="1" t="n"/>
-      <c r="I205" s="1" t="n"/>
+      <c r="H205" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I205" s="1" t="n">
+        <v>16</v>
+      </c>
       <c r="J205" s="1" t="n">
         <v>0</v>
       </c>
@@ -9085,8 +9133,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H208" s="1" t="n"/>
-      <c r="I208" s="1" t="n"/>
+      <c r="H208" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="I208" s="1" t="n">
+        <v>28</v>
+      </c>
       <c r="J208" s="1" t="n">
         <v>0</v>
       </c>
@@ -9123,8 +9175,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H209" s="1" t="n"/>
-      <c r="I209" s="1" t="n"/>
+      <c r="H209" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="I209" s="1" t="n">
+        <v>25</v>
+      </c>
       <c r="J209" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 25, 2026 - Part 5
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -8401,8 +8401,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H190" s="1" t="n"/>
-      <c r="I190" s="1" t="n"/>
+      <c r="H190" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="I190" s="1" t="n">
+        <v>30</v>
+      </c>
       <c r="J190" s="1" t="n">
         <v>0</v>
       </c>
@@ -8439,8 +8443,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H191" s="1" t="n"/>
-      <c r="I191" s="1" t="n"/>
+      <c r="H191" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I191" s="1" t="n">
+        <v>16</v>
+      </c>
       <c r="J191" s="1" t="n">
         <v>0</v>
       </c>
@@ -8813,8 +8821,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H200" s="1" t="n"/>
-      <c r="I200" s="1" t="n"/>
+      <c r="H200" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I200" s="1" t="n">
+        <v>17</v>
+      </c>
       <c r="J200" s="1" t="n">
         <v>0</v>
       </c>
@@ -8851,8 +8863,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H201" s="1" t="n"/>
-      <c r="I201" s="1" t="n"/>
+      <c r="H201" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="I201" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J201" s="1" t="n">
         <v>0</v>
       </c>
@@ -9301,8 +9317,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H212" s="1" t="n"/>
-      <c r="I212" s="1" t="n"/>
+      <c r="H212" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="I212" s="1" t="n">
+        <v>35</v>
+      </c>
       <c r="J212" s="1" t="n">
         <v>0</v>
       </c>
@@ -9339,8 +9359,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H213" s="1" t="n"/>
-      <c r="I213" s="1" t="n"/>
+      <c r="H213" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="I213" s="1" t="n">
+        <v>21</v>
+      </c>
       <c r="J213" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 25, 2026 - Part 6
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -9073,8 +9073,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H206" s="1" t="n"/>
-      <c r="I206" s="1" t="n"/>
+      <c r="H206" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I206" s="1" t="n">
+        <v>3</v>
+      </c>
       <c r="J206" s="1" t="n">
         <v>0</v>
       </c>
@@ -9111,8 +9115,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H207" s="1" t="n"/>
-      <c r="I207" s="1" t="n"/>
+      <c r="H207" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I207" s="1" t="n">
+        <v>20</v>
+      </c>
       <c r="J207" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 26, 2026 - Part 3
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -9409,8 +9409,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H214" s="1" t="n"/>
-      <c r="I214" s="1" t="n"/>
+      <c r="H214" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="I214" s="1" t="n">
+        <v>38</v>
+      </c>
       <c r="J214" s="1" t="n">
         <v>0</v>
       </c>
@@ -9447,8 +9451,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H215" s="1" t="n"/>
-      <c r="I215" s="1" t="n"/>
+      <c r="H215" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="I215" s="1" t="n">
+        <v>21</v>
+      </c>
       <c r="J215" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Added NFL Results for Oct 29, 2026 - Part 1
</commit_message>
<xml_diff>
--- a/DBs/nfl/Results/NFL_2026_Results.xlsx
+++ b/DBs/nfl/Results/NFL_2026_Results.xlsx
@@ -9493,8 +9493,12 @@
           <t>H</t>
         </is>
       </c>
-      <c r="H216" s="1" t="n"/>
-      <c r="I216" s="1" t="n"/>
+      <c r="H216" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="I216" s="1" t="n">
+        <v>19</v>
+      </c>
       <c r="J216" s="1" t="n">
         <v>0</v>
       </c>
@@ -9531,8 +9535,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H217" s="1" t="n"/>
-      <c r="I217" s="1" t="n"/>
+      <c r="H217" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="I217" s="1" t="n">
+        <v>27</v>
+      </c>
       <c r="J217" s="1" t="n">
         <v>0</v>
       </c>

</xml_diff>